<commit_message>
inclui EDP CPFL Itau XP e pagina de negociacoes
</commit_message>
<xml_diff>
--- a/reports/relatorio_2026_01.xlsx
+++ b/reports/relatorio_2026_01.xlsx
@@ -417,14 +417,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="31" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="47" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -463,26 +463,82 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GRUPO KAZA JACAREÍ</t>
+          <t>XP Investimentos</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
+          <t>17/01/2026</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>dados incompletos</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>cronograma &amp; negociação casa_Jacareí</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>downloads\pdfs\2026\Cronograma_venda casa_Jacarei.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CPFL</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>R$ 286,91</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>28/01/2026</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>extraido corpo email</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Conta por e-mail CPFL - Protocolo: 0385467621</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GRUPO KAZA JACAREÍ</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>30/01/2026</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>dados incompletos</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Extrato de aluguel de locação</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>downloads\pdfs\2026\8591_0_9_3_7684666530_extrato_grupokaza.pdf</t>
         </is>

</xml_diff>